<commit_message>
data: refresh 2026-10-27 19:02 UTC
</commit_message>
<xml_diff>
--- a/data/h8-quarterly.xlsx
+++ b/data/h8-quarterly.xlsx
@@ -7359,23 +7359,23 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>17640.27</v>
+        <v>17615.1</v>
       </c>
       <c r="G47" t="n">
         <v>1.83</v>
       </c>
       <c r="H47" t="n">
-        <v>3.93</v>
+        <v>3.95</v>
       </c>
       <c r="I47" t="n">
         <v>3</v>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>17784.17</v>
+        <v>17758.47</v>
       </c>
       <c r="L47" t="n">
-        <v>2.24</v>
+        <v>2.25</v>
       </c>
       <c r="M47" t="n">
         <v>3.3</v>
@@ -7385,87 +7385,83 @@
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
-        <v>17913.07</v>
+        <v>17886.23</v>
       </c>
       <c r="Q47" t="n">
         <v>3.03</v>
       </c>
       <c r="R47" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="S47" t="n">
         <v>3</v>
       </c>
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="n">
-        <v>18058.3</v>
+        <v>18031.4</v>
       </c>
       <c r="V47" t="n">
         <v>3.36</v>
       </c>
       <c r="W47" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
       <c r="X47" t="n">
         <v>3</v>
       </c>
       <c r="Y47" t="inlineStr"/>
       <c r="Z47" t="n">
-        <v>18207.57</v>
+        <v>18181.03</v>
       </c>
       <c r="AA47" t="n">
-        <v>3.22</v>
+        <v>3.21</v>
       </c>
       <c r="AB47" t="n">
-        <v>3.35</v>
+        <v>3.36</v>
       </c>
       <c r="AC47" t="n">
         <v>3</v>
       </c>
       <c r="AD47" t="inlineStr"/>
       <c r="AE47" t="n">
-        <v>18461.47</v>
+        <v>18435.07</v>
       </c>
       <c r="AF47" t="n">
         <v>3.81</v>
       </c>
       <c r="AG47" t="n">
-        <v>5.7</v>
+        <v>5.71</v>
       </c>
       <c r="AH47" t="n">
         <v>3</v>
       </c>
       <c r="AI47" t="inlineStr"/>
       <c r="AJ47" t="n">
-        <v>18797.33</v>
+        <v>18769.53</v>
       </c>
       <c r="AK47" t="n">
         <v>4.94</v>
       </c>
       <c r="AL47" t="n">
-        <v>7.48</v>
+        <v>7.46</v>
       </c>
       <c r="AM47" t="n">
         <v>3</v>
       </c>
       <c r="AN47" t="inlineStr"/>
       <c r="AO47" t="n">
-        <v>19058.4</v>
+        <v>19075.13</v>
       </c>
       <c r="AP47" t="n">
-        <v>5.54</v>
+        <v>5.79</v>
       </c>
       <c r="AQ47" t="n">
-        <v>5.67</v>
+        <v>6.67</v>
       </c>
       <c r="AR47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS47" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AS47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7494,7 +7490,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>5404.43</v>
+        <v>5401.57</v>
       </c>
       <c r="G48" t="n">
         <v>8.33</v>
@@ -7507,100 +7503,96 @@
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>5525.73</v>
+        <v>5523.07</v>
       </c>
       <c r="L48" t="n">
         <v>9.35</v>
       </c>
       <c r="M48" t="n">
-        <v>9.279999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="N48" t="n">
         <v>3</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>5574.7</v>
+        <v>5571.43</v>
       </c>
       <c r="Q48" t="n">
-        <v>7.31</v>
+        <v>7.32</v>
       </c>
       <c r="R48" t="n">
-        <v>3.59</v>
+        <v>3.55</v>
       </c>
       <c r="S48" t="n">
         <v>3</v>
       </c>
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="n">
-        <v>5653.3</v>
+        <v>5649.67</v>
       </c>
       <c r="V48" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="W48" t="n">
-        <v>5.76</v>
+        <v>5.74</v>
       </c>
       <c r="X48" t="n">
         <v>3</v>
       </c>
       <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="n">
-        <v>6191.63</v>
+        <v>6188.3</v>
       </c>
       <c r="AA48" t="n">
-        <v>14.57</v>
+        <v>14.56</v>
       </c>
       <c r="AB48" t="n">
-        <v>43.88</v>
+        <v>43.94</v>
       </c>
       <c r="AC48" t="n">
         <v>3</v>
       </c>
       <c r="AD48" t="inlineStr"/>
       <c r="AE48" t="n">
-        <v>6751.43</v>
+        <v>6748.17</v>
       </c>
       <c r="AF48" t="n">
         <v>22.18</v>
       </c>
       <c r="AG48" t="n">
-        <v>41.37</v>
+        <v>41.4</v>
       </c>
       <c r="AH48" t="n">
         <v>3</v>
       </c>
       <c r="AI48" t="inlineStr"/>
       <c r="AJ48" t="n">
-        <v>6935.87</v>
+        <v>6935.47</v>
       </c>
       <c r="AK48" t="n">
-        <v>24.42</v>
+        <v>24.48</v>
       </c>
       <c r="AL48" t="n">
-        <v>11.38</v>
+        <v>11.57</v>
       </c>
       <c r="AM48" t="n">
         <v>3</v>
       </c>
       <c r="AN48" t="inlineStr"/>
       <c r="AO48" t="n">
-        <v>7107.9</v>
+        <v>7146.83</v>
       </c>
       <c r="AP48" t="n">
-        <v>25.73</v>
+        <v>26.5</v>
       </c>
       <c r="AQ48" t="n">
-        <v>10.3</v>
+        <v>12.76</v>
       </c>
       <c r="AR48" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS48" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AS48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -7629,46 +7621,46 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>10647.63</v>
+        <v>10631.53</v>
       </c>
       <c r="G49" t="n">
         <v>-1.28</v>
       </c>
       <c r="H49" t="n">
-        <v>3.35</v>
+        <v>3.39</v>
       </c>
       <c r="I49" t="n">
         <v>3</v>
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>10705.2</v>
+        <v>10688.37</v>
       </c>
       <c r="L49" t="n">
         <v>-0.14</v>
       </c>
       <c r="M49" t="n">
-        <v>2.18</v>
+        <v>2.16</v>
       </c>
       <c r="N49" t="n">
         <v>3</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
-        <v>10807.7</v>
+        <v>10790.4</v>
       </c>
       <c r="Q49" t="n">
-        <v>2.24</v>
+        <v>2.22</v>
       </c>
       <c r="R49" t="n">
-        <v>3.89</v>
+        <v>3.87</v>
       </c>
       <c r="S49" t="n">
         <v>3</v>
       </c>
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="n">
-        <v>10878.73</v>
+        <v>10861.5</v>
       </c>
       <c r="V49" t="n">
         <v>3.02</v>
@@ -7681,61 +7673,57 @@
       </c>
       <c r="Y49" t="inlineStr"/>
       <c r="Z49" t="n">
-        <v>10503.43</v>
+        <v>10486.53</v>
       </c>
       <c r="AA49" t="n">
-        <v>-1.35</v>
+        <v>-1.36</v>
       </c>
       <c r="AB49" t="n">
-        <v>-13.1</v>
+        <v>-13.11</v>
       </c>
       <c r="AC49" t="n">
         <v>3</v>
       </c>
       <c r="AD49" t="inlineStr"/>
       <c r="AE49" t="n">
-        <v>10210.83</v>
+        <v>10193.67</v>
       </c>
       <c r="AF49" t="n">
-        <v>-4.62</v>
+        <v>-4.63</v>
       </c>
       <c r="AG49" t="n">
-        <v>-10.69</v>
+        <v>-10.71</v>
       </c>
       <c r="AH49" t="n">
         <v>3</v>
       </c>
       <c r="AI49" t="inlineStr"/>
       <c r="AJ49" t="n">
-        <v>10359.1</v>
+        <v>10338.17</v>
       </c>
       <c r="AK49" t="n">
-        <v>-4.15</v>
+        <v>-4.19</v>
       </c>
       <c r="AL49" t="n">
-        <v>5.94</v>
+        <v>5.79</v>
       </c>
       <c r="AM49" t="n">
         <v>3</v>
       </c>
       <c r="AN49" t="inlineStr"/>
       <c r="AO49" t="n">
-        <v>10444.5</v>
+        <v>10427.27</v>
       </c>
       <c r="AP49" t="n">
-        <v>-3.99</v>
+        <v>-4</v>
       </c>
       <c r="AQ49" t="n">
-        <v>3.34</v>
+        <v>3.49</v>
       </c>
       <c r="AR49" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS49" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AS49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -7764,113 +7752,109 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1588.2</v>
+        <v>1582</v>
       </c>
       <c r="G50" t="n">
         <v>2.57</v>
       </c>
       <c r="H50" t="n">
-        <v>-10.11</v>
+        <v>-10.2</v>
       </c>
       <c r="I50" t="n">
         <v>3</v>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>1553.23</v>
+        <v>1547.03</v>
       </c>
       <c r="L50" t="n">
-        <v>-4.16</v>
+        <v>-4.19</v>
       </c>
       <c r="M50" t="n">
-        <v>-8.52</v>
+        <v>-8.550000000000001</v>
       </c>
       <c r="N50" t="n">
         <v>3</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
-        <v>1530.67</v>
+        <v>1524.4</v>
       </c>
       <c r="Q50" t="n">
-        <v>-5.5</v>
+        <v>-5.52</v>
       </c>
       <c r="R50" t="n">
-        <v>-5.69</v>
+        <v>-5.72</v>
       </c>
       <c r="S50" t="n">
         <v>3</v>
       </c>
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="n">
-        <v>1526.27</v>
+        <v>1520.23</v>
       </c>
       <c r="V50" t="n">
-        <v>-6.43</v>
+        <v>-6.45</v>
       </c>
       <c r="W50" t="n">
-        <v>-1.14</v>
+        <v>-1.09</v>
       </c>
       <c r="X50" t="n">
         <v>3</v>
       </c>
       <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="n">
-        <v>1512.5</v>
+        <v>1506.2</v>
       </c>
       <c r="AA50" t="n">
-        <v>-4.77</v>
+        <v>-4.79</v>
       </c>
       <c r="AB50" t="n">
-        <v>-3.56</v>
+        <v>-3.64</v>
       </c>
       <c r="AC50" t="n">
         <v>3</v>
       </c>
       <c r="AD50" t="inlineStr"/>
       <c r="AE50" t="n">
-        <v>1499.2</v>
+        <v>1493.23</v>
       </c>
       <c r="AF50" t="n">
         <v>-3.48</v>
       </c>
       <c r="AG50" t="n">
-        <v>-3.47</v>
+        <v>-3.4</v>
       </c>
       <c r="AH50" t="n">
         <v>3</v>
       </c>
       <c r="AI50" t="inlineStr"/>
       <c r="AJ50" t="n">
-        <v>1502.37</v>
+        <v>1495.9</v>
       </c>
       <c r="AK50" t="n">
-        <v>-1.85</v>
+        <v>-1.87</v>
       </c>
       <c r="AL50" t="n">
-        <v>0.85</v>
+        <v>0.72</v>
       </c>
       <c r="AM50" t="n">
         <v>3</v>
       </c>
       <c r="AN50" t="inlineStr"/>
       <c r="AO50" t="n">
-        <v>1506</v>
+        <v>1501.03</v>
       </c>
       <c r="AP50" t="n">
-        <v>-1.33</v>
+        <v>-1.26</v>
       </c>
       <c r="AQ50" t="n">
-        <v>0.97</v>
+        <v>1.38</v>
       </c>
       <c r="AR50" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS50" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AS50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -7990,22 +7974,18 @@
       </c>
       <c r="AN51" t="inlineStr"/>
       <c r="AO51" t="n">
-        <v>3063.35</v>
+        <v>3070.57</v>
       </c>
       <c r="AP51" t="n">
-        <v>5.37</v>
+        <v>5.62</v>
       </c>
       <c r="AQ51" t="n">
-        <v>5.49</v>
+        <v>6.49</v>
       </c>
       <c r="AR51" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS51" t="inlineStr">
-        <is>
-          <t>QTD</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="AS51" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">

</xml_diff>